<commit_message>
Updated peer review documentation
</commit_message>
<xml_diff>
--- a/peer_review/20260519_du_jufe_dm_peer_review_01_selected_vector_student.xlsx
+++ b/peer_review/20260519_du_jufe_dm_peer_review_01_selected_vector_student.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rpi\source\20260512_du_jufe_dm\20260512_du_jufe_dm_rpi\peer_review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8598047B-1C65-4AEC-8786-C5C0B154386D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1BFE3B3-EE76-416F-BC71-43B7DB7654D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Learning Targets" sheetId="1" r:id="rId1"/>
@@ -233,12 +233,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -881,28 +880,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="22" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="23" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="24" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="25" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="26" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="27" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="28" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="29" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="31" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="32" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="33" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="34" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="35" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="36" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="37" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="38" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="39" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="40" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="41" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="42" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="33" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="34" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="35" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="36" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="37" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="38" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="39" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="40" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="41" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="42" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>